<commit_message>
Actualización Historial y para Bitacora
</commit_message>
<xml_diff>
--- a/assets/Historico.xlsx
+++ b/assets/Historico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SUBDIRECCIÓN\Desarrollo Docente\APROVECHAMIENTO ACADEMICO\TABLERO-DOCENTE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F923FF-6325-45C9-AE14-E296801A4AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43BF7D37-34A4-47EA-96DF-F959D8F185D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16371" yWindow="0" windowWidth="16629" windowHeight="17880" xr2:uid="{E296F2EF-5FA4-4C61-B291-B758F5755367}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="16629" windowHeight="17880" xr2:uid="{E296F2EF-5FA4-4C61-B291-B758F5755367}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="1" r:id="rId1"/>
@@ -945,6 +945,9 @@
       <c r="L8">
         <v>59.1</v>
       </c>
+      <c r="M8">
+        <v>34.700000000000003</v>
+      </c>
       <c r="N8">
         <v>18.75</v>
       </c>
@@ -971,6 +974,9 @@
       <c r="L9">
         <v>149</v>
       </c>
+      <c r="M9">
+        <v>139</v>
+      </c>
       <c r="N9">
         <v>69</v>
       </c>
@@ -982,6 +988,9 @@
       <c r="B10" t="s">
         <v>64</v>
       </c>
+      <c r="L10">
+        <v>7.4</v>
+      </c>
       <c r="M10">
         <v>11</v>
       </c>
@@ -1302,6 +1311,9 @@
       <c r="L20">
         <v>75.900000000000006</v>
       </c>
+      <c r="M20">
+        <v>90.4</v>
+      </c>
       <c r="N20">
         <v>87.97</v>
       </c>
@@ -1328,6 +1340,9 @@
       <c r="L21">
         <v>264</v>
       </c>
+      <c r="M21">
+        <v>311</v>
+      </c>
       <c r="N21">
         <v>351</v>
       </c>
@@ -1659,6 +1674,9 @@
       <c r="L32">
         <v>61.6</v>
       </c>
+      <c r="M32">
+        <v>88.8</v>
+      </c>
       <c r="N32">
         <v>92.84</v>
       </c>
@@ -1685,6 +1703,9 @@
       <c r="L33">
         <v>151</v>
       </c>
+      <c r="M33">
+        <v>237</v>
+      </c>
       <c r="N33">
         <v>337</v>
       </c>
@@ -2016,6 +2037,9 @@
       <c r="L44">
         <v>93.5</v>
       </c>
+      <c r="M44">
+        <v>90.5</v>
+      </c>
       <c r="N44">
         <v>72.19</v>
       </c>
@@ -2042,6 +2066,9 @@
       <c r="L45">
         <v>259</v>
       </c>
+      <c r="M45">
+        <v>219</v>
+      </c>
       <c r="N45">
         <v>218</v>
       </c>
@@ -2373,6 +2400,9 @@
       <c r="L56">
         <v>46.9</v>
       </c>
+      <c r="M56">
+        <v>56.3</v>
+      </c>
       <c r="N56">
         <v>27.89</v>
       </c>
@@ -2399,6 +2429,9 @@
       <c r="L57">
         <v>136</v>
       </c>
+      <c r="M57">
+        <v>211</v>
+      </c>
       <c r="N57">
         <v>99</v>
       </c>
@@ -2730,6 +2763,9 @@
       <c r="L68">
         <v>65</v>
       </c>
+      <c r="M68">
+        <v>61.5</v>
+      </c>
       <c r="N68">
         <v>68.7</v>
       </c>
@@ -2756,6 +2792,9 @@
       <c r="L69">
         <v>104</v>
       </c>
+      <c r="M69">
+        <v>134</v>
+      </c>
       <c r="N69">
         <v>169</v>
       </c>
@@ -3087,6 +3126,9 @@
       <c r="L80">
         <v>99</v>
       </c>
+      <c r="M80">
+        <v>53.1</v>
+      </c>
       <c r="N80">
         <v>80.540000000000006</v>
       </c>
@@ -3113,6 +3155,9 @@
       <c r="L81">
         <v>308</v>
       </c>
+      <c r="M81">
+        <v>144</v>
+      </c>
       <c r="N81">
         <v>269</v>
       </c>
@@ -3444,6 +3489,9 @@
       <c r="L92">
         <v>50.4</v>
       </c>
+      <c r="M92">
+        <v>41.2</v>
+      </c>
       <c r="N92">
         <v>53</v>
       </c>
@@ -3470,6 +3518,9 @@
       <c r="L93">
         <v>202</v>
       </c>
+      <c r="M93">
+        <v>243</v>
+      </c>
       <c r="N93">
         <v>285</v>
       </c>
@@ -3801,6 +3852,9 @@
       <c r="L104">
         <v>57.6</v>
       </c>
+      <c r="M104">
+        <v>47.8</v>
+      </c>
       <c r="N104">
         <v>27.8</v>
       </c>
@@ -3827,6 +3881,9 @@
       <c r="L105">
         <v>366</v>
       </c>
+      <c r="M105">
+        <v>382</v>
+      </c>
       <c r="N105">
         <v>228</v>
       </c>
@@ -4158,6 +4215,9 @@
       <c r="L116">
         <v>82.3</v>
       </c>
+      <c r="M116">
+        <v>90.9</v>
+      </c>
       <c r="N116">
         <v>76.39</v>
       </c>
@@ -4184,6 +4244,9 @@
       <c r="L117">
         <v>135</v>
       </c>
+      <c r="M117">
+        <v>210</v>
+      </c>
       <c r="N117">
         <v>178</v>
       </c>
@@ -4515,6 +4578,9 @@
       <c r="L128">
         <v>86.7</v>
       </c>
+      <c r="M128">
+        <v>98</v>
+      </c>
       <c r="N128">
         <v>98.7</v>
       </c>
@@ -4541,6 +4607,9 @@
       <c r="L129">
         <v>299</v>
       </c>
+      <c r="M129">
+        <v>300</v>
+      </c>
       <c r="N129">
         <v>379</v>
       </c>
@@ -4872,6 +4941,9 @@
       <c r="L140">
         <v>47.1</v>
       </c>
+      <c r="M140">
+        <v>83.8</v>
+      </c>
       <c r="N140">
         <v>79.5</v>
       </c>
@@ -4898,6 +4970,9 @@
       <c r="L141">
         <v>130</v>
       </c>
+      <c r="M141">
+        <v>201</v>
+      </c>
       <c r="N141">
         <v>221</v>
       </c>
@@ -5229,6 +5304,9 @@
       <c r="L152">
         <v>88.6</v>
       </c>
+      <c r="M152">
+        <v>60.6</v>
+      </c>
       <c r="N152">
         <v>56.53</v>
       </c>
@@ -5255,6 +5333,9 @@
       <c r="L153">
         <v>226</v>
       </c>
+      <c r="M153">
+        <v>215</v>
+      </c>
       <c r="N153">
         <v>277</v>
       </c>
@@ -5586,6 +5667,9 @@
       <c r="L164">
         <v>53.5</v>
       </c>
+      <c r="M164">
+        <v>79.8</v>
+      </c>
       <c r="N164">
         <v>64.14</v>
       </c>
@@ -5612,6 +5696,9 @@
       <c r="L165">
         <v>99</v>
       </c>
+      <c r="M165">
+        <v>134</v>
+      </c>
       <c r="N165">
         <v>127</v>
       </c>
@@ -5943,6 +6030,9 @@
       <c r="L176">
         <v>94.7</v>
       </c>
+      <c r="M176">
+        <v>93.9</v>
+      </c>
       <c r="N176">
         <v>85.62</v>
       </c>
@@ -5969,6 +6059,9 @@
       <c r="L177">
         <v>125</v>
       </c>
+      <c r="M177">
+        <v>138</v>
+      </c>
       <c r="N177">
         <v>131</v>
       </c>
@@ -6300,6 +6393,9 @@
       <c r="L188">
         <v>92.2</v>
       </c>
+      <c r="M188">
+        <v>71.900000000000006</v>
+      </c>
       <c r="N188">
         <v>81.52</v>
       </c>
@@ -6326,6 +6422,9 @@
       <c r="L189">
         <v>402</v>
       </c>
+      <c r="M189">
+        <v>282</v>
+      </c>
       <c r="N189">
         <v>375</v>
       </c>
@@ -6657,6 +6756,9 @@
       <c r="L200">
         <v>71.8</v>
       </c>
+      <c r="M200">
+        <v>49.6</v>
+      </c>
       <c r="N200">
         <v>66.209999999999994</v>
       </c>
@@ -6683,6 +6785,9 @@
       <c r="L201">
         <v>191</v>
       </c>
+      <c r="M201">
+        <v>176</v>
+      </c>
       <c r="N201">
         <v>241</v>
       </c>
@@ -7014,6 +7119,9 @@
       <c r="L212">
         <v>83</v>
       </c>
+      <c r="M212">
+        <v>82.6</v>
+      </c>
       <c r="N212">
         <v>66.44</v>
       </c>
@@ -7040,6 +7148,9 @@
       <c r="L213">
         <v>409</v>
       </c>
+      <c r="M213">
+        <v>542</v>
+      </c>
       <c r="N213">
         <v>394</v>
       </c>
@@ -7371,6 +7482,9 @@
       <c r="L224">
         <v>81.8</v>
       </c>
+      <c r="M224">
+        <v>65.3</v>
+      </c>
       <c r="N224">
         <v>52.96</v>
       </c>
@@ -7397,6 +7511,9 @@
       <c r="L225">
         <v>171</v>
       </c>
+      <c r="M225">
+        <v>160</v>
+      </c>
       <c r="N225">
         <v>152</v>
       </c>
@@ -7728,6 +7845,9 @@
       <c r="L236">
         <v>64.3</v>
       </c>
+      <c r="M236">
+        <v>65.400000000000006</v>
+      </c>
       <c r="N236">
         <v>63.1</v>
       </c>
@@ -7754,6 +7874,9 @@
       <c r="L237">
         <v>187</v>
       </c>
+      <c r="M237">
+        <v>189</v>
+      </c>
       <c r="N237">
         <v>277</v>
       </c>
@@ -8085,6 +8208,9 @@
       <c r="L248">
         <v>61.8</v>
       </c>
+      <c r="M248">
+        <v>53</v>
+      </c>
       <c r="N248">
         <v>45.01</v>
       </c>
@@ -8111,6 +8237,9 @@
       <c r="L249">
         <v>223</v>
       </c>
+      <c r="M249">
+        <v>221</v>
+      </c>
       <c r="N249">
         <v>194</v>
       </c>
@@ -8442,6 +8571,9 @@
       <c r="L260">
         <v>65.900000000000006</v>
       </c>
+      <c r="M260">
+        <v>78.099999999999994</v>
+      </c>
       <c r="N260">
         <v>84.77</v>
       </c>
@@ -8468,6 +8600,9 @@
       <c r="L261">
         <v>213</v>
       </c>
+      <c r="M261">
+        <v>325</v>
+      </c>
       <c r="N261">
         <v>384</v>
       </c>
@@ -8479,18 +8614,6 @@
       <c r="B262" t="s">
         <v>64</v>
       </c>
-      <c r="H262">
-        <v>34.799999999999997</v>
-      </c>
-      <c r="I262">
-        <v>23.8</v>
-      </c>
-      <c r="J262">
-        <v>17.5</v>
-      </c>
-      <c r="K262">
-        <v>17.399999999999999</v>
-      </c>
       <c r="M262">
         <v>7.4</v>
       </c>
@@ -8811,6 +8934,9 @@
       <c r="L272">
         <v>43.3</v>
       </c>
+      <c r="M272">
+        <v>69.7</v>
+      </c>
       <c r="N272">
         <v>59.52</v>
       </c>
@@ -8837,6 +8963,9 @@
       <c r="L273">
         <v>127</v>
       </c>
+      <c r="M273">
+        <v>253</v>
+      </c>
       <c r="N273">
         <v>225</v>
       </c>
@@ -8848,18 +8977,6 @@
       <c r="B274" t="s">
         <v>64</v>
       </c>
-      <c r="H274">
-        <v>21.9</v>
-      </c>
-      <c r="I274">
-        <v>20.399999999999999</v>
-      </c>
-      <c r="J274">
-        <v>12.6</v>
-      </c>
-      <c r="K274">
-        <v>10.9</v>
-      </c>
       <c r="M274">
         <v>11.2</v>
       </c>
@@ -9180,6 +9297,9 @@
       <c r="L284">
         <v>50.4</v>
       </c>
+      <c r="M284">
+        <v>54.8</v>
+      </c>
       <c r="N284">
         <v>8.74</v>
       </c>
@@ -9206,6 +9326,9 @@
       <c r="L285">
         <v>192</v>
       </c>
+      <c r="M285">
+        <v>242</v>
+      </c>
       <c r="N285">
         <v>36</v>
       </c>
@@ -9217,18 +9340,6 @@
       <c r="B286" t="s">
         <v>64</v>
       </c>
-      <c r="H286">
-        <v>26.7</v>
-      </c>
-      <c r="I286">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="J286">
-        <v>0.8</v>
-      </c>
-      <c r="K286">
-        <v>3.1</v>
-      </c>
       <c r="M286">
         <v>4.4000000000000004</v>
       </c>
@@ -9549,6 +9660,9 @@
       <c r="L296">
         <v>87.6</v>
       </c>
+      <c r="M296">
+        <v>59.3</v>
+      </c>
       <c r="N296">
         <v>59.09</v>
       </c>
@@ -9575,6 +9689,9 @@
       <c r="L297">
         <v>220</v>
       </c>
+      <c r="M297">
+        <v>143</v>
+      </c>
       <c r="N297">
         <v>143</v>
       </c>
@@ -9586,18 +9703,6 @@
       <c r="B298" t="s">
         <v>64</v>
       </c>
-      <c r="H298">
-        <v>37.4</v>
-      </c>
-      <c r="I298">
-        <v>1.5</v>
-      </c>
-      <c r="J298">
-        <v>0.5</v>
-      </c>
-      <c r="K298">
-        <v>6.9</v>
-      </c>
       <c r="M298">
         <v>6</v>
       </c>
@@ -9918,6 +10023,9 @@
       <c r="L308">
         <v>55.8</v>
       </c>
+      <c r="M308">
+        <v>58</v>
+      </c>
       <c r="N308">
         <v>61.13</v>
       </c>
@@ -9944,6 +10052,9 @@
       <c r="L309">
         <v>148</v>
       </c>
+      <c r="M309">
+        <v>207</v>
+      </c>
       <c r="N309">
         <v>228</v>
       </c>
@@ -9955,18 +10066,6 @@
       <c r="B310" t="s">
         <v>64</v>
       </c>
-      <c r="H310">
-        <v>37.299999999999997</v>
-      </c>
-      <c r="I310">
-        <v>13.9</v>
-      </c>
-      <c r="J310">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="K310">
-        <v>8</v>
-      </c>
       <c r="M310">
         <v>7.1</v>
       </c>
@@ -10287,6 +10386,9 @@
       <c r="L320">
         <v>77.5</v>
       </c>
+      <c r="M320">
+        <v>37.200000000000003</v>
+      </c>
       <c r="N320">
         <v>57.88</v>
       </c>
@@ -10313,6 +10415,9 @@
       <c r="L321">
         <v>290</v>
       </c>
+      <c r="M321">
+        <v>148</v>
+      </c>
       <c r="N321">
         <v>312</v>
       </c>
@@ -10324,18 +10429,6 @@
       <c r="B322" t="s">
         <v>64</v>
       </c>
-      <c r="H322">
-        <v>34.799999999999997</v>
-      </c>
-      <c r="I322">
-        <v>19.399999999999999</v>
-      </c>
-      <c r="J322">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="K322">
-        <v>10.7</v>
-      </c>
       <c r="M322">
         <v>8.8000000000000007</v>
       </c>
@@ -10656,6 +10749,9 @@
       <c r="L332">
         <v>83.8</v>
       </c>
+      <c r="M332">
+        <v>61.5</v>
+      </c>
       <c r="N332">
         <v>50.18</v>
       </c>
@@ -10682,6 +10778,9 @@
       <c r="L333">
         <v>238</v>
       </c>
+      <c r="M333">
+        <v>184</v>
+      </c>
       <c r="N333">
         <v>136</v>
       </c>
@@ -10693,18 +10792,6 @@
       <c r="B334" t="s">
         <v>64</v>
       </c>
-      <c r="H334">
-        <v>35.799999999999997</v>
-      </c>
-      <c r="I334">
-        <v>11.1</v>
-      </c>
-      <c r="J334">
-        <v>3.4</v>
-      </c>
-      <c r="K334">
-        <v>4.3</v>
-      </c>
       <c r="M334">
         <v>6.5</v>
       </c>
@@ -11025,6 +11112,9 @@
       <c r="L344">
         <v>51</v>
       </c>
+      <c r="M344">
+        <v>71.599999999999994</v>
+      </c>
       <c r="N344">
         <v>82.92</v>
       </c>
@@ -11051,6 +11141,9 @@
       <c r="L345">
         <v>77</v>
       </c>
+      <c r="M345">
+        <v>96</v>
+      </c>
       <c r="N345">
         <v>199</v>
       </c>
@@ -11062,18 +11155,6 @@
       <c r="B346" t="s">
         <v>64</v>
       </c>
-      <c r="H346">
-        <v>27.5</v>
-      </c>
-      <c r="I346">
-        <v>13.2</v>
-      </c>
-      <c r="J346">
-        <v>5.6</v>
-      </c>
-      <c r="K346">
-        <v>8.9</v>
-      </c>
       <c r="M346">
         <v>10.9</v>
       </c>
@@ -11394,6 +11475,9 @@
       <c r="L356">
         <v>71.099999999999994</v>
       </c>
+      <c r="M356">
+        <v>96.4</v>
+      </c>
       <c r="N356">
         <v>92.06</v>
       </c>
@@ -11420,6 +11504,9 @@
       <c r="L357">
         <v>271</v>
       </c>
+      <c r="M357">
+        <v>264</v>
+      </c>
       <c r="N357">
         <v>290</v>
       </c>
@@ -11431,18 +11518,6 @@
       <c r="B358" t="s">
         <v>64</v>
       </c>
-      <c r="H358">
-        <v>35</v>
-      </c>
-      <c r="I358">
-        <v>0.2</v>
-      </c>
-      <c r="J358">
-        <v>1</v>
-      </c>
-      <c r="K358">
-        <v>5.9</v>
-      </c>
       <c r="M358">
         <v>9.8000000000000007</v>
       </c>
@@ -11763,6 +11838,9 @@
       <c r="L368">
         <v>66.5</v>
       </c>
+      <c r="M368">
+        <v>82.5</v>
+      </c>
       <c r="N368">
         <v>57.58</v>
       </c>
@@ -11789,6 +11867,9 @@
       <c r="L369">
         <v>308</v>
       </c>
+      <c r="M369">
+        <v>415</v>
+      </c>
       <c r="N369">
         <v>304</v>
       </c>
@@ -11800,18 +11881,6 @@
       <c r="B370" t="s">
         <v>64</v>
       </c>
-      <c r="H370">
-        <v>17.100000000000001</v>
-      </c>
-      <c r="I370">
-        <v>17.600000000000001</v>
-      </c>
-      <c r="J370">
-        <v>11.5</v>
-      </c>
-      <c r="K370">
-        <v>6.7</v>
-      </c>
       <c r="M370">
         <v>9.1</v>
       </c>
@@ -12132,6 +12201,9 @@
       <c r="L380">
         <v>93.5</v>
       </c>
+      <c r="M380">
+        <v>100</v>
+      </c>
       <c r="N380">
         <v>98.73</v>
       </c>
@@ -12158,6 +12230,9 @@
       <c r="L381">
         <v>144</v>
       </c>
+      <c r="M381">
+        <v>167</v>
+      </c>
       <c r="N381">
         <v>155</v>
       </c>
@@ -12169,18 +12244,6 @@
       <c r="B382" t="s">
         <v>64</v>
       </c>
-      <c r="H382">
-        <v>25.8</v>
-      </c>
-      <c r="I382">
-        <v>2.5</v>
-      </c>
-      <c r="J382">
-        <v>4.8</v>
-      </c>
-      <c r="K382">
-        <v>7</v>
-      </c>
       <c r="M382">
         <v>7.4</v>
       </c>
@@ -12501,6 +12564,9 @@
       <c r="L392">
         <v>21.3</v>
       </c>
+      <c r="M392">
+        <v>56</v>
+      </c>
       <c r="N392">
         <v>38.26</v>
       </c>
@@ -12527,6 +12593,9 @@
       <c r="L393">
         <v>26</v>
       </c>
+      <c r="M393">
+        <v>65</v>
+      </c>
       <c r="N393">
         <v>44</v>
       </c>
@@ -12538,18 +12607,6 @@
       <c r="B394" t="s">
         <v>64</v>
       </c>
-      <c r="H394">
-        <v>40.9</v>
-      </c>
-      <c r="I394">
-        <v>8</v>
-      </c>
-      <c r="J394">
-        <v>3.6</v>
-      </c>
-      <c r="K394">
-        <v>4.8</v>
-      </c>
       <c r="M394">
         <v>11.5</v>
       </c>
@@ -12870,6 +12927,9 @@
       <c r="L404">
         <v>71.599999999999994</v>
       </c>
+      <c r="M404">
+        <v>85.5</v>
+      </c>
       <c r="N404">
         <v>80.25</v>
       </c>
@@ -12896,6 +12956,9 @@
       <c r="L405">
         <v>126</v>
       </c>
+      <c r="M405">
+        <v>112</v>
+      </c>
       <c r="N405">
         <v>130</v>
       </c>
@@ -12907,18 +12970,6 @@
       <c r="B406" t="s">
         <v>64</v>
       </c>
-      <c r="H406">
-        <v>33.299999999999997</v>
-      </c>
-      <c r="I406">
-        <v>20.8</v>
-      </c>
-      <c r="J406">
-        <v>8.5</v>
-      </c>
-      <c r="K406">
-        <v>12.9</v>
-      </c>
       <c r="M406">
         <v>18.899999999999999</v>
       </c>
@@ -13239,6 +13290,9 @@
       <c r="L416">
         <v>73.2</v>
       </c>
+      <c r="M416">
+        <v>64.3</v>
+      </c>
       <c r="N416">
         <v>0.88</v>
       </c>
@@ -13265,6 +13319,9 @@
       <c r="L417">
         <v>112</v>
       </c>
+      <c r="M417">
+        <v>169</v>
+      </c>
       <c r="N417">
         <v>2</v>
       </c>
@@ -13276,18 +13333,6 @@
       <c r="B418" t="s">
         <v>64</v>
       </c>
-      <c r="H418">
-        <v>62.2</v>
-      </c>
-      <c r="I418">
-        <v>13.4</v>
-      </c>
-      <c r="J418">
-        <v>7.8</v>
-      </c>
-      <c r="K418">
-        <v>8.9</v>
-      </c>
       <c r="M418">
         <v>8.3000000000000007</v>
       </c>
@@ -13608,6 +13653,9 @@
       <c r="L428">
         <v>74.8</v>
       </c>
+      <c r="M428">
+        <v>83.9</v>
+      </c>
       <c r="N428">
         <v>74.430000000000007</v>
       </c>
@@ -13634,6 +13682,9 @@
       <c r="L429">
         <v>306</v>
       </c>
+      <c r="M429">
+        <v>392</v>
+      </c>
       <c r="N429">
         <v>390</v>
       </c>
@@ -13965,6 +14016,9 @@
       <c r="L440">
         <v>45.9</v>
       </c>
+      <c r="M440">
+        <v>58.6</v>
+      </c>
       <c r="N440">
         <v>52.92</v>
       </c>
@@ -13991,6 +14045,9 @@
       <c r="L441">
         <v>113</v>
       </c>
+      <c r="M441">
+        <v>146</v>
+      </c>
       <c r="N441">
         <v>181</v>
       </c>
@@ -14322,6 +14379,9 @@
       <c r="L452">
         <v>82.3</v>
       </c>
+      <c r="M452">
+        <v>90.1</v>
+      </c>
       <c r="N452">
         <v>90.06</v>
       </c>
@@ -14348,6 +14408,9 @@
       <c r="L453">
         <v>102</v>
       </c>
+      <c r="M453">
+        <v>118</v>
+      </c>
       <c r="N453">
         <v>154</v>
       </c>
@@ -14679,6 +14742,9 @@
       <c r="L464">
         <v>80.099999999999994</v>
       </c>
+      <c r="M464">
+        <v>73.7</v>
+      </c>
       <c r="N464">
         <v>45.09</v>
       </c>
@@ -14705,6 +14771,9 @@
       <c r="L465">
         <v>185</v>
       </c>
+      <c r="M465">
+        <v>216</v>
+      </c>
       <c r="N465">
         <v>156</v>
       </c>
@@ -15036,6 +15105,9 @@
       <c r="L476">
         <v>69.599999999999994</v>
       </c>
+      <c r="M476">
+        <v>67.3</v>
+      </c>
       <c r="N476">
         <v>63.1</v>
       </c>
@@ -15061,6 +15133,9 @@
       </c>
       <c r="L477">
         <v>7734</v>
+      </c>
+      <c r="M477">
+        <v>8450</v>
       </c>
       <c r="N477">
         <v>8440</v>

</xml_diff>